<commit_message>
paper: address review and package latex report
</commit_message>
<xml_diff>
--- a/outputs/submission/q2_fhv_pricing.xlsx
+++ b/outputs/submission/q2_fhv_pricing.xlsx
@@ -2056,10 +2056,10 @@
         <v>15.89</v>
       </c>
       <c r="Y18" t="n">
-        <v>5.981000000000002</v>
+        <v>5.981</v>
       </c>
       <c r="Z18" t="n">
-        <v>0.6035926935109499</v>
+        <v>0.6035926935109496</v>
       </c>
     </row>
     <row r="19">
@@ -2146,10 +2146,10 @@
         <v>15.28</v>
       </c>
       <c r="Y19" t="n">
-        <v>4.534249999999998</v>
+        <v>4.53425</v>
       </c>
       <c r="Z19" t="n">
-        <v>0.4219575180885464</v>
+        <v>0.4219575180885467</v>
       </c>
     </row>
     <row r="20">
@@ -2850,10 +2850,10 @@
         <v>9.470000000000001</v>
       </c>
       <c r="Y27" t="n">
-        <v>3.701500000000001</v>
+        <v>3.7015</v>
       </c>
       <c r="Z27" t="n">
-        <v>0.6416746121175352</v>
+        <v>0.6416746121175348</v>
       </c>
     </row>
     <row r="28">
@@ -3031,7 +3031,7 @@
         <v>3.028</v>
       </c>
       <c r="Z29" t="n">
-        <v>0.4558867810900332</v>
+        <v>0.455886781090033</v>
       </c>
     </row>
     <row r="30">
@@ -3734,10 +3734,10 @@
         <v>20.82</v>
       </c>
       <c r="Y37" t="n">
-        <v>7.844000000000001</v>
+        <v>7.843999999999999</v>
       </c>
       <c r="Z37" t="n">
-        <v>0.6045006165228115</v>
+        <v>0.6045006165228113</v>
       </c>
     </row>
     <row r="38">
@@ -3912,10 +3912,10 @@
         <v>9.73</v>
       </c>
       <c r="Y39" t="n">
-        <v>3.567710440003781</v>
+        <v>3.56771044000378</v>
       </c>
       <c r="Z39" t="n">
-        <v>0.5789585843489591</v>
+        <v>0.5789585843489589</v>
       </c>
     </row>
     <row r="40">
@@ -4264,10 +4264,10 @@
         <v>25.01</v>
       </c>
       <c r="Y43" t="n">
-        <v>9.283000000000005</v>
+        <v>9.282999999999999</v>
       </c>
       <c r="Z43" t="n">
-        <v>0.5902587906148664</v>
+        <v>0.5902587906148662</v>
       </c>
     </row>
     <row r="44">
@@ -5062,10 +5062,10 @@
         <v>25.98</v>
       </c>
       <c r="Y52" t="n">
-        <v>6.527000000000005</v>
+        <v>6.527000000000001</v>
       </c>
       <c r="Z52" t="n">
-        <v>0.3355266539865319</v>
+        <v>0.3355266539865317</v>
       </c>
     </row>
     <row r="53">
@@ -6299,7 +6299,7 @@
         <v>23.573</v>
       </c>
       <c r="Z66" t="n">
-        <v>0.8569818591631222</v>
+        <v>0.856981859163122</v>
       </c>
     </row>
     <row r="67">
@@ -6475,7 +6475,7 @@
         <v>3.65</v>
       </c>
       <c r="Z68" t="n">
-        <v>0.5667701863354039</v>
+        <v>0.5667701863354037</v>
       </c>
     </row>
     <row r="69">
@@ -8322,10 +8322,10 @@
         <v>22.8</v>
       </c>
       <c r="Y89" t="n">
-        <v>8.204499999999999</v>
+        <v>8.204500000000001</v>
       </c>
       <c r="Z89" t="n">
-        <v>0.5621253125963481</v>
+        <v>0.5621253125963483</v>
       </c>
     </row>
     <row r="90">
@@ -9116,10 +9116,10 @@
         <v>8.99</v>
       </c>
       <c r="Y98" t="n">
-        <v>3.176500000000001</v>
+        <v>3.1765</v>
       </c>
       <c r="Z98" t="n">
-        <v>0.5464006192483015</v>
+        <v>0.5464006192483013</v>
       </c>
     </row>
     <row r="99">
@@ -10088,10 +10088,10 @@
         <v>6.85</v>
       </c>
       <c r="Y109" t="n">
-        <v>1.785</v>
+        <v>1.784999999999999</v>
       </c>
       <c r="Z109" t="n">
-        <v>0.3524185587364265</v>
+        <v>0.3524185587364263</v>
       </c>
     </row>
     <row r="110">
@@ -10352,10 +10352,10 @@
         <v>20.92</v>
       </c>
       <c r="Y112" t="n">
-        <v>8.236500000000003</v>
+        <v>8.236500000000001</v>
       </c>
       <c r="Z112" t="n">
-        <v>0.6493869988567827</v>
+        <v>0.6493869988567825</v>
       </c>
     </row>
     <row r="113">
@@ -10440,10 +10440,10 @@
         <v>8.01</v>
       </c>
       <c r="Y113" t="n">
-        <v>2.5715</v>
+        <v>2.571499999999999</v>
       </c>
       <c r="Z113" t="n">
-        <v>0.4728325825135608</v>
+        <v>0.4728325825135606</v>
       </c>
     </row>
     <row r="114">

</xml_diff>